<commit_message>
Add character personality to 6 cases; author Boulderfield & The Weekly Rate
Gave each of this week's protagonists a distinct name and real
character texture (fixing a "three Priyas" template collision), added
visuals and glossary context to Fizzer Order per review feedback, and
authored two new reinforcement cases (Boulderfield, Pre-Algebra;
The Weekly Rate, Algebra) to round out the week's level mix after
swapping Fizzer Order and Kite Cut out of this week's release in favor
of Creek Span. All 8 cases re-verified through the full case-readiness
gate (Tier 1 + all 7 Tier 2 probes) after edits. Refreshed dashboard
and pipeline_status.json to register the 2 new cases and correct
stale stage/status data for all 8.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cases/dice-roll/published/Dice Roll - Data.xlsx
+++ b/cases/dice-roll/published/Dice Roll - Data.xlsx
@@ -478,6 +478,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -485,6 +486,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -602,6 +604,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1023,6 +1026,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1134,6 +1138,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1259,6 +1264,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>

</xml_diff>